<commit_message>
feat: add new list to test data for squares description
</commit_message>
<xml_diff>
--- a/data/test_simple.xlsx
+++ b/data/test_simple.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PetProjects\archeoplan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PetProjects\archeoplan\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB347E0-6171-495F-884C-A409ED229C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D2D7B4-72FB-49FA-8BB9-BB0F4AB13842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="массавы матэрыял 80-90" sheetId="1" r:id="rId1"/>
-    <sheet name="массавы матэрыял 70-80" sheetId="2" r:id="rId2"/>
+    <sheet name="Раскоп" sheetId="3" r:id="rId1"/>
+    <sheet name="массавы матэрыял 80-90" sheetId="1" r:id="rId2"/>
+    <sheet name="массавы матэрыял 70-80" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -412,6 +413,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{818AC747-FD02-4D1F-B815-727BD7F09210}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>451</v>
+      </c>
+      <c r="B1">
+        <v>452</v>
+      </c>
+      <c r="C1">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>448</v>
+      </c>
+      <c r="B2">
+        <v>449</v>
+      </c>
+      <c r="C2">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>445</v>
+      </c>
+      <c r="B3">
+        <v>446</v>
+      </c>
+      <c r="C3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>443</v>
+      </c>
+      <c r="B4">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>441</v>
+      </c>
+      <c r="B5">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>439</v>
+      </c>
+      <c r="B6">
+        <v>440</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -598,7 +666,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3372260-9C5C-490F-9AB2-747E128296A4}">
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>